<commit_message>
Carrie Grochow \$100 → Ben & Jack; raised \$1,485; ticker \$4,735
</commit_message>
<xml_diff>
--- a/Squeeze_Project_Donations.xlsx
+++ b/Squeeze_Project_Donations.xlsx
@@ -1463,7 +1463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1893,23 +1893,43 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="inlineStr">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Carrie Grochow</t>
+        </is>
+      </c>
+      <c r="C23" s="20" t="n">
+        <v>100</v>
+      </c>
+      <c r="D23" s="24" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C23" s="16">
+      <c r="C24" s="16">
         <f>SUM(C4:C21)</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="25" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="25" t="inlineStr">
         <is>
           <t>% of Goal</t>
         </is>
       </c>
-      <c r="C24" s="26">
+      <c r="C25" s="26">
         <f>C22/B2</f>
         <v/>
       </c>
@@ -2169,11 +2189,6 @@
           <t>Mar 25</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Eileen Linde</t>
-        </is>
-      </c>
       <c r="C13" s="20" t="n">
         <v>100</v>
       </c>

</xml_diff>

<commit_message>
Excel: clean minimal redesign, no color noise
</commit_message>
<xml_diff>
--- a/Squeeze_Project_Donations.xlsx
+++ b/Squeeze_Project_Donations.xlsx
@@ -21,11 +21,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,46 +34,29 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="14"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <color rgb="00888888"/>
+      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
     </font>
     <font>
       <b val="1"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00635BFF"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00B8860B"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="006A0DAD"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="000070BA"/>
+      <sz val="12"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -83,66 +65,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001a2e23"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002d4a3e"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="004A6FA5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00CC0000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="008B1A1A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001a2744"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F0F0F0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00444444"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F0EEFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF8E1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F5E6FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8F4FF"/>
+        <fgColor rgb="00EEEEEE"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -150,61 +77,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <top style="medium">
+        <color rgb="00999999"/>
+      </top>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00EEEEEE"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -570,207 +471,192 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The Squeeze Project — Donation Summary</t>
+          <t>The Squeeze Project — Donations</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Updated March 25, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
           <t>Ambassador</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Camp</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Total Raised</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Raised</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Goal</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>% to Goal</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>% of Goal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Luke &amp; Aria Kerman</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Camp IHC</t>
         </is>
       </c>
-      <c r="C3" s="4">
+      <c r="C5" s="4">
         <f>'Luke &amp; Aria Kerman'!C12</f>
         <v/>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D5" s="4" t="n">
         <v>2250</v>
       </c>
-      <c r="E3" s="5">
-        <f>C3/D3</f>
+      <c r="E5" s="5">
+        <f>C5/D5</f>
         <v/>
       </c>
-      <c r="F3" s="4">
-        <f>D3-C3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Tessa Forman</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Camp Pontiac</t>
         </is>
       </c>
-      <c r="C4" s="7">
+      <c r="C6" s="4">
         <f>'Tessa Forman'!C21</f>
         <v/>
       </c>
-      <c r="D4" s="7" t="n">
+      <c r="D6" s="4" t="n">
         <v>2250</v>
       </c>
-      <c r="E4" s="8">
-        <f>C4/D4</f>
-        <v/>
-      </c>
-      <c r="F4" s="7">
-        <f>D4-C4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Ben &amp; Jack</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Camp Wah-Nee</t>
-        </is>
-      </c>
-      <c r="C5" s="10">
-        <f>'Ben &amp; Jack'!C22</f>
-        <v/>
-      </c>
-      <c r="D5" s="10" t="n">
-        <v>2250</v>
-      </c>
-      <c r="E5" s="11">
-        <f>C5/D5</f>
-        <v/>
-      </c>
-      <c r="F5" s="10">
-        <f>D5-C5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Jordana Brody</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>Camp Westmont</t>
-        </is>
-      </c>
-      <c r="C6" s="13">
-        <f>'Jordana Brody'!C13</f>
-        <v/>
-      </c>
-      <c r="D6" s="13" t="n">
-        <v>2250</v>
-      </c>
-      <c r="E6" s="14">
+      <c r="E6" s="5">
         <f>C6/D6</f>
         <v/>
       </c>
-      <c r="F6" s="13">
-        <f>D6-C6</f>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ben &amp; Jack</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Camp Wah-Nee</t>
+        </is>
+      </c>
+      <c r="C7" s="4">
+        <f>'Ben &amp; Jack'!C24</f>
         <v/>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="D7" s="4" t="n">
+        <v>2250</v>
+      </c>
+      <c r="E7" s="5">
+        <f>C7/D7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Jordana Brody</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Camp Westmont</t>
+        </is>
+      </c>
+      <c r="C8" s="4">
+        <f>'Jordana Brody'!C14</f>
+        <v/>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>2250</v>
+      </c>
+      <c r="E8" s="5">
+        <f>C8/D8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Parker Wellen</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Camp Pontiac</t>
         </is>
       </c>
-      <c r="C7" s="7">
+      <c r="C9" s="4">
         <f>'Parker Wellen'!C8</f>
         <v/>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D9" s="4" t="n">
         <v>2250</v>
       </c>
-      <c r="E7" s="8">
-        <f>C7/D7</f>
+      <c r="E9" s="5">
+        <f>C9/D9</f>
         <v/>
       </c>
-      <c r="F7" s="7">
-        <f>D7-C7</f>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n"/>
+      <c r="C11" s="8">
+        <f>SUM(C5:C9)</f>
         <v/>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="15" t="inlineStr">
-        <is>
-          <t>GRAND TOTAL</t>
-        </is>
-      </c>
-      <c r="C8" s="16">
-        <f>SUM(C3:C7)</f>
+      <c r="D11" s="9" t="n">
+        <v>11250</v>
+      </c>
+      <c r="E11" s="10">
+        <f>C11/D11</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -781,247 +667,218 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Luke &amp; Aria Kerman — Camp IHC</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Goal:</t>
-        </is>
-      </c>
-      <c r="B2" s="18" t="n">
-        <v>2250</v>
-      </c>
-    </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B3" s="19" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Donor</t>
         </is>
       </c>
-      <c r="C3" s="19" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="D3" s="19" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="E3" s="19" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>jayson@license-2-play.com</t>
         </is>
       </c>
-      <c r="C4" s="20" t="n">
+      <c r="C4" s="13" t="n">
         <v>500</v>
       </c>
-      <c r="D4" s="21" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Jarret Kerman</t>
         </is>
       </c>
-      <c r="C5" s="20" t="n">
+      <c r="C5" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="D5" s="21" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Brooke Jung</t>
         </is>
       </c>
-      <c r="C6" s="20" t="n">
+      <c r="C6" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="D6" s="21" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Melanie Ringold</t>
         </is>
       </c>
-      <c r="C7" s="20" t="n">
+      <c r="C7" s="13" t="n">
         <v>54</v>
       </c>
-      <c r="D7" s="21" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Jarret Kerman</t>
         </is>
       </c>
-      <c r="C8" s="20" t="n">
+      <c r="C8" s="13" t="n">
         <v>200</v>
       </c>
-      <c r="D8" s="21" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Von Maur Foundation</t>
         </is>
       </c>
-      <c r="C9" s="20" t="n">
+      <c r="C9" s="13" t="n">
         <v>250</v>
       </c>
-      <c r="D9" s="22" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>David Brown</t>
         </is>
       </c>
-      <c r="C10" s="20" t="n">
+      <c r="C10" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="D10" s="23" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Zelle</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Craig Brown</t>
         </is>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="13" t="n">
         <v>50</v>
       </c>
-      <c r="D11" s="24" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="7" t="n"/>
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C12" s="16">
+      <c r="C12" s="8">
         <f>SUM(C4:C11)</f>
         <v/>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="25" t="inlineStr">
-        <is>
-          <t>% of Goal</t>
-        </is>
-      </c>
-      <c r="C13" s="26">
-        <f>C12/B2</f>
-        <v/>
-      </c>
+      <c r="D12" s="7" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A12:B12"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1032,427 +889,398 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="27" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Tessa Forman — Camp Pontiac</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Goal:</t>
-        </is>
-      </c>
-      <c r="B2" s="18" t="n">
-        <v>2250</v>
-      </c>
-    </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B3" s="19" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Donor</t>
         </is>
       </c>
-      <c r="C3" s="19" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="D3" s="19" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="E3" s="19" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Allison Slansky</t>
         </is>
       </c>
-      <c r="C4" s="20" t="n">
+      <c r="C4" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="D4" s="24" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Annabelle Greenberg</t>
         </is>
       </c>
-      <c r="C5" s="20" t="n">
+      <c r="C5" s="13" t="n">
         <v>15</v>
       </c>
-      <c r="D5" s="24" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Joshua Henkel</t>
         </is>
       </c>
-      <c r="C6" s="20" t="n">
+      <c r="C6" s="13" t="n">
         <v>36</v>
       </c>
-      <c r="D6" s="24" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Jen Seiden</t>
         </is>
       </c>
-      <c r="C7" s="20" t="n">
+      <c r="C7" s="13" t="n">
         <v>36</v>
       </c>
-      <c r="D7" s="24" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Robyn Kreiner</t>
         </is>
       </c>
-      <c r="C8" s="20" t="n">
+      <c r="C8" s="13" t="n">
         <v>36</v>
       </c>
-      <c r="D8" s="24" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Erica Polavieja</t>
         </is>
       </c>
-      <c r="C9" s="20" t="n">
+      <c r="C9" s="13" t="n">
         <v>50</v>
       </c>
-      <c r="D9" s="24" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Marissa Drogin</t>
         </is>
       </c>
-      <c r="C10" s="20" t="n">
+      <c r="C10" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="D10" s="24" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Cori Zummo</t>
         </is>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="D11" s="24" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Lindsey Schnepper</t>
         </is>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="D12" s="24" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Christine Schwartz</t>
         </is>
       </c>
-      <c r="C13" s="20" t="n">
+      <c r="C13" s="13" t="n">
         <v>50</v>
       </c>
-      <c r="D13" s="21" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>sarimskier@gmail.com</t>
         </is>
       </c>
-      <c r="C14" s="20" t="n">
+      <c r="C14" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="D14" s="21" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Jen Schwartz</t>
         </is>
       </c>
-      <c r="C15" s="20" t="n">
+      <c r="C15" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="D15" s="24" t="inlineStr">
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Tracy Paley</t>
         </is>
       </c>
-      <c r="C16" s="20" t="n">
+      <c r="C16" s="13" t="n">
         <v>50</v>
       </c>
-      <c r="D16" s="21" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>masetheace728@icloud.com</t>
         </is>
       </c>
-      <c r="C17" s="20" t="n">
+      <c r="C17" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="D17" s="21" t="inlineStr">
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>Stage to Screen</t>
         </is>
       </c>
-      <c r="C18" s="20" t="n">
+      <c r="C18" s="13" t="n">
         <v>250</v>
       </c>
-      <c r="D18" s="22" t="inlineStr">
+      <c r="D18" s="12" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>Rose</t>
         </is>
       </c>
-      <c r="C19" s="20" t="n">
+      <c r="C19" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="D19" s="22" t="inlineStr">
+      <c r="D19" s="12" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>Rose</t>
         </is>
       </c>
-      <c r="C20" s="20" t="n">
+      <c r="C20" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="D20" s="22" t="inlineStr">
+      <c r="D20" s="12" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="inlineStr">
+      <c r="A21" s="7" t="n"/>
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C21" s="16">
+      <c r="C21" s="8">
         <f>SUM(C4:C20)</f>
         <v/>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="25" t="inlineStr">
-        <is>
-          <t>% of Goal</t>
-        </is>
-      </c>
-      <c r="C22" s="26">
-        <f>C21/B2</f>
-        <v/>
-      </c>
+      <c r="D21" s="7" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1463,482 +1291,458 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="28" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Ben &amp; Jack — Camp Wah-Nee</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Goal:</t>
-        </is>
-      </c>
-      <c r="B2" s="18" t="n">
-        <v>2250</v>
-      </c>
-    </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B3" s="19" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Donor</t>
         </is>
       </c>
-      <c r="C3" s="19" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="D3" s="19" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="E3" s="19" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Jayson Siano</t>
         </is>
       </c>
-      <c r="C4" s="20" t="n">
+      <c r="C4" s="13" t="n">
         <v>200</v>
       </c>
-      <c r="D4" s="21" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Jessica Zipkin</t>
         </is>
       </c>
-      <c r="C5" s="20" t="n">
+      <c r="C5" s="13" t="n">
         <v>150</v>
       </c>
-      <c r="D5" s="24" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Stephanie Barilan</t>
         </is>
       </c>
-      <c r="C6" s="20" t="n">
+      <c r="C6" s="13" t="n">
         <v>150</v>
       </c>
-      <c r="D6" s="24" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Evane Klein</t>
         </is>
       </c>
-      <c r="C7" s="20" t="n">
+      <c r="C7" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="D7" s="24" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Dana Block</t>
         </is>
       </c>
-      <c r="C8" s="20" t="n">
+      <c r="C8" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="D8" s="24" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Jessica Goldstein</t>
         </is>
       </c>
-      <c r="C9" s="20" t="n">
+      <c r="C9" s="13" t="n">
         <v>50</v>
       </c>
-      <c r="D9" s="24" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Jessica Greenwald</t>
         </is>
       </c>
-      <c r="C10" s="20" t="n">
+      <c r="C10" s="13" t="n">
         <v>50</v>
       </c>
-      <c r="D10" s="24" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Jaclyn Vida</t>
         </is>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="13" t="n">
         <v>50</v>
       </c>
-      <c r="D11" s="24" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Alyse Stern</t>
         </is>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="13" t="n">
         <v>50</v>
       </c>
-      <c r="D12" s="24" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>ali horowitz</t>
         </is>
       </c>
-      <c r="C13" s="20" t="n">
+      <c r="C13" s="13" t="n">
         <v>50</v>
       </c>
-      <c r="D13" s="24" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>Dina Goldberg</t>
         </is>
       </c>
-      <c r="C14" s="20" t="n">
+      <c r="C14" s="13" t="n">
         <v>50</v>
       </c>
-      <c r="D14" s="24" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Liz Beler</t>
         </is>
       </c>
-      <c r="C15" s="20" t="n">
+      <c r="C15" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="D15" s="24" t="inlineStr">
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Elizabeth Zorn</t>
         </is>
       </c>
-      <c r="C16" s="20" t="n">
+      <c r="C16" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="D16" s="24" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>Michael Jacobson</t>
         </is>
       </c>
-      <c r="C17" s="20" t="n">
+      <c r="C17" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="D17" s="24" t="inlineStr">
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>Erica Oliver</t>
         </is>
       </c>
-      <c r="C18" s="20" t="n">
+      <c r="C18" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="D18" s="24" t="inlineStr">
+      <c r="D18" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>Robyn Sachnoff</t>
         </is>
       </c>
-      <c r="C19" s="20" t="n">
+      <c r="C19" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="D19" s="24" t="inlineStr">
+      <c r="D19" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>Jennifer Brogadir</t>
         </is>
       </c>
-      <c r="C20" s="20" t="n">
+      <c r="C20" s="13" t="n">
         <v>20</v>
       </c>
-      <c r="D20" s="24" t="inlineStr">
+      <c r="D20" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>Ellen Jacobson</t>
         </is>
       </c>
-      <c r="C21" s="20" t="n">
+      <c r="C21" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="D21" s="24" t="inlineStr">
+      <c r="D21" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="C22" s="20" t="n">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Joey Stella</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="n">
         <v>200</v>
       </c>
-      <c r="D22" s="24" t="inlineStr">
+      <c r="D22" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>Carrie Grochow</t>
         </is>
       </c>
-      <c r="C23" s="20" t="n">
+      <c r="C23" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="D23" s="24" t="inlineStr">
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="inlineStr">
+      <c r="A24" s="7" t="n"/>
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C24" s="16">
-        <f>SUM(C4:C21)</f>
+      <c r="C24" s="8">
+        <f>SUM(C4:C23)</f>
         <v/>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="25" t="inlineStr">
-        <is>
-          <t>% of Goal</t>
-        </is>
-      </c>
-      <c r="C25" s="26">
-        <f>C22/B2</f>
-        <v/>
-      </c>
+      <c r="D24" s="7" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A22:B22"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1949,282 +1753,258 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="29" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Jordana Brody — Camp Westmont</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Goal:</t>
-        </is>
-      </c>
-      <c r="B2" s="18" t="n">
-        <v>2250</v>
-      </c>
-    </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B3" s="19" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Donor</t>
         </is>
       </c>
-      <c r="C3" s="19" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="D3" s="19" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="E3" s="19" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Evan Krakauer</t>
         </is>
       </c>
-      <c r="C4" s="20" t="n">
+      <c r="C4" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="D4" s="24" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>hallie polsky</t>
         </is>
       </c>
-      <c r="C5" s="20" t="n">
+      <c r="C5" s="13" t="n">
         <v>36</v>
       </c>
-      <c r="D5" s="24" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Alexa Scalzi</t>
         </is>
       </c>
-      <c r="C6" s="20" t="n">
+      <c r="C6" s="13" t="n">
         <v>30</v>
       </c>
-      <c r="D6" s="24" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Jaimee Manger</t>
         </is>
       </c>
-      <c r="C7" s="20" t="n">
+      <c r="C7" s="13" t="n">
         <v>20</v>
       </c>
-      <c r="D7" s="24" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Karen Ganz</t>
         </is>
       </c>
-      <c r="C8" s="20" t="n">
+      <c r="C8" s="13" t="n">
         <v>18</v>
       </c>
-      <c r="D8" s="24" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Debbi Kauffman</t>
         </is>
       </c>
-      <c r="C9" s="20" t="n">
+      <c r="C9" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="D9" s="24" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Jan Mirman</t>
         </is>
       </c>
-      <c r="C10" s="20" t="n">
+      <c r="C10" s="13" t="n">
         <v>50</v>
       </c>
-      <c r="D10" s="24" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Beth Brody</t>
         </is>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="D11" s="24" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Steve Kreinik</t>
         </is>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="13" t="n">
         <v>250</v>
       </c>
-      <c r="D12" s="23" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Zelle</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="C13" s="20" t="n">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Eileen Linde</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="D13" s="24" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="7" t="n"/>
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C14" s="16">
-        <f>SUM(C4:C12)</f>
+      <c r="C14" s="8">
+        <f>SUM(C4:C13)</f>
         <v/>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="25" t="inlineStr">
-        <is>
-          <t>% of Goal</t>
-        </is>
-      </c>
-      <c r="C15" s="26">
-        <f>C13/B2</f>
-        <v/>
-      </c>
+      <c r="D14" s="7" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2235,167 +2015,138 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="27" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Parker Wellen — Camp Pontiac</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Goal:</t>
-        </is>
-      </c>
-      <c r="B2" s="18" t="n">
-        <v>2250</v>
-      </c>
-    </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B3" s="19" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Donor</t>
         </is>
       </c>
-      <c r="C3" s="19" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="D3" s="19" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="E3" s="19" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Jason Hornig</t>
         </is>
       </c>
-      <c r="C4" s="20" t="n">
+      <c r="C4" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="D4" s="24" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Meredith Wellen</t>
         </is>
       </c>
-      <c r="C5" s="20" t="n">
+      <c r="C5" s="13" t="n">
         <v>36</v>
       </c>
-      <c r="D5" s="24" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Meredith Wellen</t>
         </is>
       </c>
-      <c r="C6" s="20" t="n">
+      <c r="C6" s="13" t="n">
         <v>50</v>
       </c>
-      <c r="D6" s="24" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Lindsay Koonin</t>
         </is>
       </c>
-      <c r="C7" s="20" t="n">
+      <c r="C7" s="13" t="n">
         <v>118</v>
       </c>
-      <c r="D7" s="24" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="7" t="n"/>
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C8" s="16">
+      <c r="C8" s="8">
         <f>SUM(C4:C7)</f>
         <v/>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="25" t="inlineStr">
-        <is>
-          <t>% of Goal</t>
-        </is>
-      </c>
-      <c r="C9" s="26">
-        <f>C8/B2</f>
-        <v/>
-      </c>
+      <c r="D8" s="7" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add fee estimates to admin page and Excel
</commit_message>
<xml_diff>
--- a/Squeeze_Project_Donations.xlsx
+++ b/Squeeze_Project_Donations.xlsx
@@ -24,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,6 +50,10 @@
     <font>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00888888"/>
     </font>
   </fonts>
   <fills count="3">
@@ -87,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -102,6 +106,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -467,14 +475,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -487,7 +497,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Updated March 25, 2026</t>
+          <t>Fee rates: Venmo 1.9% + $0.10 · Stripe 2.9% + $0.30 · Check/Zelle free</t>
         </is>
       </c>
     </row>
@@ -504,15 +514,25 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Raised</t>
+          <t>Gross Raised</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
+          <t>Est. Fees</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Net Received</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
           <t>Goal</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>% to Goal</t>
         </is>
@@ -533,11 +553,19 @@
         <f>'Luke &amp; Aria Kerman'!C12</f>
         <v/>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="4">
+        <f>'Luke &amp; Aria Kerman'!C13</f>
+        <v/>
+      </c>
+      <c r="E5" s="4">
+        <f>'Luke &amp; Aria Kerman'!C14</f>
+        <v/>
+      </c>
+      <c r="F5" s="4" t="n">
         <v>2250</v>
       </c>
-      <c r="E5" s="5">
-        <f>C5/D5</f>
+      <c r="G5" s="5">
+        <f>C5/F5</f>
         <v/>
       </c>
     </row>
@@ -556,11 +584,19 @@
         <f>'Tessa Forman'!C21</f>
         <v/>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="4">
+        <f>'Tessa Forman'!C22</f>
+        <v/>
+      </c>
+      <c r="E6" s="4">
+        <f>'Tessa Forman'!C23</f>
+        <v/>
+      </c>
+      <c r="F6" s="4" t="n">
         <v>2250</v>
       </c>
-      <c r="E6" s="5">
-        <f>C6/D6</f>
+      <c r="G6" s="5">
+        <f>C6/F6</f>
         <v/>
       </c>
     </row>
@@ -576,14 +612,22 @@
         </is>
       </c>
       <c r="C7" s="4">
-        <f>'Ben &amp; Jack'!C24</f>
-        <v/>
-      </c>
-      <c r="D7" s="4" t="n">
+        <f>'Ben &amp; Jack'!C25</f>
+        <v/>
+      </c>
+      <c r="D7" s="4">
+        <f>'Ben &amp; Jack'!C26</f>
+        <v/>
+      </c>
+      <c r="E7" s="4">
+        <f>'Ben &amp; Jack'!C27</f>
+        <v/>
+      </c>
+      <c r="F7" s="4" t="n">
         <v>2250</v>
       </c>
-      <c r="E7" s="5">
-        <f>C7/D7</f>
+      <c r="G7" s="5">
+        <f>C7/F7</f>
         <v/>
       </c>
     </row>
@@ -602,11 +646,19 @@
         <f>'Jordana Brody'!C14</f>
         <v/>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="4">
+        <f>'Jordana Brody'!C15</f>
+        <v/>
+      </c>
+      <c r="E8" s="4">
+        <f>'Jordana Brody'!C16</f>
+        <v/>
+      </c>
+      <c r="F8" s="4" t="n">
         <v>2250</v>
       </c>
-      <c r="E8" s="5">
-        <f>C8/D8</f>
+      <c r="G8" s="5">
+        <f>C8/F8</f>
         <v/>
       </c>
     </row>
@@ -625,11 +677,19 @@
         <f>'Parker Wellen'!C8</f>
         <v/>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" s="4">
+        <f>'Parker Wellen'!C9</f>
+        <v/>
+      </c>
+      <c r="E9" s="4">
+        <f>'Parker Wellen'!C10</f>
+        <v/>
+      </c>
+      <c r="F9" s="4" t="n">
         <v>2250</v>
       </c>
-      <c r="E9" s="5">
-        <f>C9/D9</f>
+      <c r="G9" s="5">
+        <f>C9/F9</f>
         <v/>
       </c>
     </row>
@@ -644,11 +704,19 @@
         <f>SUM(C5:C9)</f>
         <v/>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="9">
+        <f>SUM(D5:D9)</f>
+        <v/>
+      </c>
+      <c r="E11" s="8">
+        <f>SUM(E5:E9)</f>
+        <v/>
+      </c>
+      <c r="F11" s="9" t="n">
         <v>11250</v>
       </c>
-      <c r="E11" s="10">
-        <f>C11/D11</f>
+      <c r="G11" s="10">
+        <f>C11/F11</f>
         <v/>
       </c>
     </row>
@@ -663,13 +731,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -679,45 +748,37 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Fees: Venmo 1.9%+$0.10 · Stripe 2.9%+$0.30 · Check/Zelle free</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Donor</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Mar 24</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>jayson@license-2-play.com</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="n">
-        <v>500</v>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>Stripe</t>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Est. Fee</t>
         </is>
       </c>
     </row>
@@ -729,36 +790,42 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Jarret Kerman</t>
+          <t>jayson@license-2-play.com</t>
         </is>
       </c>
       <c r="C5" s="13" t="n">
-        <v>10</v>
+        <v>500</v>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>14.8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>Mar 25</t>
+          <t>Mar 24</t>
         </is>
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>Brooke Jung</t>
+          <t>Jarret Kerman</t>
         </is>
       </c>
       <c r="C6" s="13" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>0.59</v>
       </c>
     </row>
     <row r="7">
@@ -769,16 +836,19 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Melanie Ringold</t>
+          <t>Brooke Jung</t>
         </is>
       </c>
       <c r="C7" s="13" t="n">
-        <v>54</v>
+        <v>100</v>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
+      </c>
+      <c r="E7" s="13" t="n">
+        <v>3.2</v>
       </c>
     </row>
     <row r="8">
@@ -789,16 +859,19 @@
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>Jarret Kerman</t>
+          <t>Melanie Ringold</t>
         </is>
       </c>
       <c r="C8" s="13" t="n">
-        <v>200</v>
+        <v>54</v>
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
+      </c>
+      <c r="E8" s="13" t="n">
+        <v>1.87</v>
       </c>
     </row>
     <row r="9">
@@ -809,16 +882,19 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Von Maur Foundation</t>
+          <t>Jarret Kerman</t>
         </is>
       </c>
       <c r="C9" s="13" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Check</t>
-        </is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>6.1</v>
       </c>
     </row>
     <row r="10">
@@ -829,16 +905,19 @@
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>David Brown</t>
+          <t>Von Maur Foundation</t>
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>Zelle</t>
-        </is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -849,30 +928,82 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
+          <t>David Brown</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Zelle</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
           <t>Craig Brown</t>
         </is>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C12" s="13" t="n">
         <v>50</v>
       </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="n">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n"/>
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C12" s="8">
-        <f>SUM(C4:C11)</f>
-        <v/>
-      </c>
-      <c r="D12" s="7" t="n"/>
+      <c r="C13" s="8">
+        <f>SUM(C5:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="9">
+        <f>SUM(E5:E12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>Est. Fees</t>
+        </is>
+      </c>
+      <c r="C14" s="15">
+        <f>-E13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Net Received</t>
+        </is>
+      </c>
+      <c r="C15" s="17">
+        <f>C13+C14</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -885,13 +1016,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -901,45 +1033,37 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Fees: Venmo 1.9%+$0.10 · Stripe 2.9%+$0.30 · Check/Zelle free</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Donor</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Mar 24</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>Allison Slansky</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="n">
-        <v>25</v>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Est. Fee</t>
         </is>
       </c>
     </row>
@@ -951,16 +1075,19 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Annabelle Greenberg</t>
+          <t>Allison Slansky</t>
         </is>
       </c>
       <c r="C5" s="13" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>0.57</v>
       </c>
     </row>
     <row r="6">
@@ -971,16 +1098,19 @@
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>Joshua Henkel</t>
+          <t>Annabelle Greenberg</t>
         </is>
       </c>
       <c r="C6" s="13" t="n">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>0.39</v>
       </c>
     </row>
     <row r="7">
@@ -991,7 +1121,7 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Jen Seiden</t>
+          <t>Joshua Henkel</t>
         </is>
       </c>
       <c r="C7" s="13" t="n">
@@ -1002,6 +1132,9 @@
           <t>Venmo</t>
         </is>
       </c>
+      <c r="E7" s="13" t="n">
+        <v>0.78</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -1011,7 +1144,7 @@
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>Robyn Kreiner</t>
+          <t>Jen Seiden</t>
         </is>
       </c>
       <c r="C8" s="13" t="n">
@@ -1022,6 +1155,9 @@
           <t>Venmo</t>
         </is>
       </c>
+      <c r="E8" s="13" t="n">
+        <v>0.78</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -1031,16 +1167,19 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Erica Polavieja</t>
+          <t>Robyn Kreiner</t>
         </is>
       </c>
       <c r="C9" s="13" t="n">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>0.78</v>
       </c>
     </row>
     <row r="10">
@@ -1051,16 +1190,19 @@
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>Marissa Drogin</t>
+          <t>Erica Polavieja</t>
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E10" s="13" t="n">
+        <v>1.05</v>
       </c>
     </row>
     <row r="11">
@@ -1071,7 +1213,7 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Cori Zummo</t>
+          <t>Marissa Drogin</t>
         </is>
       </c>
       <c r="C11" s="13" t="n">
@@ -1082,6 +1224,9 @@
           <t>Venmo</t>
         </is>
       </c>
+      <c r="E11" s="13" t="n">
+        <v>0.57</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -1091,16 +1236,19 @@
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>Lindsey Schnepper</t>
+          <t>Cori Zummo</t>
         </is>
       </c>
       <c r="C12" s="13" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E12" s="13" t="n">
+        <v>0.57</v>
       </c>
     </row>
     <row r="13">
@@ -1111,16 +1259,19 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Christine Schwartz</t>
+          <t>Lindsey Schnepper</t>
         </is>
       </c>
       <c r="C13" s="13" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Stripe</t>
-        </is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1131,36 +1282,42 @@
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>sarimskier@gmail.com</t>
+          <t>Christine Schwartz</t>
         </is>
       </c>
       <c r="C14" s="13" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
+      </c>
+      <c r="E14" s="13" t="n">
+        <v>1.75</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>Mar 25</t>
+          <t>Mar 24</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Jen Schwartz</t>
+          <t>sarimskier@gmail.com</t>
         </is>
       </c>
       <c r="C15" s="13" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Venmo</t>
-        </is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="n">
+        <v>1.03</v>
       </c>
     </row>
     <row r="16">
@@ -1171,16 +1328,19 @@
       </c>
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t>Tracy Paley</t>
+          <t>Jen Schwartz</t>
         </is>
       </c>
       <c r="C16" s="13" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
-          <t>Stripe</t>
-        </is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -1191,16 +1351,19 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>masetheace728@icloud.com</t>
+          <t>Tracy Paley</t>
         </is>
       </c>
       <c r="C17" s="13" t="n">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
+      </c>
+      <c r="E17" s="13" t="n">
+        <v>1.75</v>
       </c>
     </row>
     <row r="18">
@@ -1211,16 +1374,19 @@
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>Stage to Screen</t>
+          <t>masetheace728@icloud.com</t>
         </is>
       </c>
       <c r="C18" s="13" t="n">
-        <v>250</v>
+        <v>5</v>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>Check</t>
-        </is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="n">
+        <v>0.45</v>
       </c>
     </row>
     <row r="19">
@@ -1231,16 +1397,19 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Rose</t>
+          <t>Stage to Screen</t>
         </is>
       </c>
       <c r="C19" s="13" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
+      </c>
+      <c r="E19" s="13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -1262,19 +1431,71 @@
           <t>Check</t>
         </is>
       </c>
+      <c r="E20" s="13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="n"/>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>Rose</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="n"/>
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C21" s="8">
-        <f>SUM(C4:C20)</f>
-        <v/>
-      </c>
-      <c r="D21" s="7" t="n"/>
+      <c r="C22" s="8">
+        <f>SUM(C5:C21)</f>
+        <v/>
+      </c>
+      <c r="D22" s="7" t="n"/>
+      <c r="E22" s="9">
+        <f>SUM(E5:E21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Est. Fees</t>
+        </is>
+      </c>
+      <c r="C23" s="15">
+        <f>-E22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>Net Received</t>
+        </is>
+      </c>
+      <c r="C24" s="17">
+        <f>C22+C23</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1287,13 +1508,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -1303,46 +1525,37 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Fees: Venmo 1.9%+$0.10 · Stripe 2.9%+$0.30 · Check/Zelle free</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Donor</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>Jayson Siano</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="n">
-        <v>200</v>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>Stripe</t>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Est. Fee</t>
         </is>
       </c>
     </row>
@@ -1354,16 +1567,19 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Jessica Zipkin</t>
+          <t>Jayson Siano</t>
         </is>
       </c>
       <c r="C5" s="13" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Venmo</t>
-        </is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>6.1</v>
       </c>
     </row>
     <row r="6">
@@ -1374,7 +1590,7 @@
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>Stephanie Barilan</t>
+          <t>Jessica Zipkin</t>
         </is>
       </c>
       <c r="C6" s="13" t="n">
@@ -1385,6 +1601,9 @@
           <t>Venmo</t>
         </is>
       </c>
+      <c r="E6" s="13" t="n">
+        <v>2.95</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -1394,16 +1613,19 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Evane Klein</t>
+          <t>Stephanie Barilan</t>
         </is>
       </c>
       <c r="C7" s="13" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E7" s="13" t="n">
+        <v>2.95</v>
       </c>
     </row>
     <row r="8">
@@ -1414,7 +1636,7 @@
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>Dana Block</t>
+          <t>Evane Klein</t>
         </is>
       </c>
       <c r="C8" s="13" t="n">
@@ -1425,6 +1647,9 @@
           <t>Venmo</t>
         </is>
       </c>
+      <c r="E8" s="13" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -1434,16 +1659,19 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Jessica Goldstein</t>
+          <t>Dana Block</t>
         </is>
       </c>
       <c r="C9" s="13" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1454,7 +1682,7 @@
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>Jessica Greenwald</t>
+          <t>Jessica Goldstein</t>
         </is>
       </c>
       <c r="C10" s="13" t="n">
@@ -1465,6 +1693,9 @@
           <t>Venmo</t>
         </is>
       </c>
+      <c r="E10" s="13" t="n">
+        <v>1.05</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -1474,7 +1705,7 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Jaclyn Vida</t>
+          <t>Jessica Greenwald</t>
         </is>
       </c>
       <c r="C11" s="13" t="n">
@@ -1485,6 +1716,9 @@
           <t>Venmo</t>
         </is>
       </c>
+      <c r="E11" s="13" t="n">
+        <v>1.05</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -1494,7 +1728,7 @@
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>Alyse Stern</t>
+          <t>Jaclyn Vida</t>
         </is>
       </c>
       <c r="C12" s="13" t="n">
@@ -1505,6 +1739,9 @@
           <t>Venmo</t>
         </is>
       </c>
+      <c r="E12" s="13" t="n">
+        <v>1.05</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
@@ -1514,7 +1751,7 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>ali horowitz</t>
+          <t>Alyse Stern</t>
         </is>
       </c>
       <c r="C13" s="13" t="n">
@@ -1525,6 +1762,9 @@
           <t>Venmo</t>
         </is>
       </c>
+      <c r="E13" s="13" t="n">
+        <v>1.05</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
@@ -1534,7 +1774,7 @@
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>Dina Goldberg</t>
+          <t>ali horowitz</t>
         </is>
       </c>
       <c r="C14" s="13" t="n">
@@ -1545,6 +1785,9 @@
           <t>Venmo</t>
         </is>
       </c>
+      <c r="E14" s="13" t="n">
+        <v>1.05</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -1554,16 +1797,19 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Liz Beler</t>
+          <t>Dina Goldberg</t>
         </is>
       </c>
       <c r="C15" s="13" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E15" s="13" t="n">
+        <v>1.05</v>
       </c>
     </row>
     <row r="16">
@@ -1574,16 +1820,19 @@
       </c>
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t>Elizabeth Zorn</t>
+          <t>Liz Beler</t>
         </is>
       </c>
       <c r="C16" s="13" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E16" s="13" t="n">
+        <v>0.86</v>
       </c>
     </row>
     <row r="17">
@@ -1594,7 +1843,7 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Michael Jacobson</t>
+          <t>Elizabeth Zorn</t>
         </is>
       </c>
       <c r="C17" s="13" t="n">
@@ -1605,6 +1854,9 @@
           <t>Venmo</t>
         </is>
       </c>
+      <c r="E17" s="13" t="n">
+        <v>0.57</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
@@ -1614,7 +1866,7 @@
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>Erica Oliver</t>
+          <t>Michael Jacobson</t>
         </is>
       </c>
       <c r="C18" s="13" t="n">
@@ -1625,6 +1877,9 @@
           <t>Venmo</t>
         </is>
       </c>
+      <c r="E18" s="13" t="n">
+        <v>0.57</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
@@ -1634,7 +1889,7 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Robyn Sachnoff</t>
+          <t>Erica Oliver</t>
         </is>
       </c>
       <c r="C19" s="13" t="n">
@@ -1645,6 +1900,9 @@
           <t>Venmo</t>
         </is>
       </c>
+      <c r="E19" s="13" t="n">
+        <v>0.57</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
@@ -1654,16 +1912,19 @@
       </c>
       <c r="B20" s="12" t="inlineStr">
         <is>
-          <t>Jennifer Brogadir</t>
+          <t>Robyn Sachnoff</t>
         </is>
       </c>
       <c r="C20" s="13" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E20" s="13" t="n">
+        <v>0.57</v>
       </c>
     </row>
     <row r="21">
@@ -1674,16 +1935,19 @@
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>Ellen Jacobson</t>
+          <t>Jennifer Brogadir</t>
         </is>
       </c>
       <c r="C21" s="13" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E21" s="13" t="n">
+        <v>0.48</v>
       </c>
     </row>
     <row r="22">
@@ -1694,16 +1958,19 @@
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>Joey Stella</t>
+          <t>Ellen Jacobson</t>
         </is>
       </c>
       <c r="C22" s="13" t="n">
-        <v>200</v>
+        <v>25</v>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E22" s="13" t="n">
+        <v>0.57</v>
       </c>
     </row>
     <row r="23">
@@ -1714,16 +1981,19 @@
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Carrie Grochow</t>
+          <t>Joey Stella</t>
         </is>
       </c>
       <c r="C23" s="13" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E23" s="13" t="n">
+        <v>3.9</v>
       </c>
     </row>
     <row r="24">
@@ -1734,7 +2004,7 @@
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>Rebecca Brogadir</t>
+          <t>Carrie Grochow</t>
         </is>
       </c>
       <c r="C24" s="13" t="n">
@@ -1745,19 +2015,71 @@
           <t>Venmo</t>
         </is>
       </c>
+      <c r="E24" s="13" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="n"/>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>Rebecca Brogadir</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="n"/>
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C25" s="8">
-        <f>SUM(C4:C23)</f>
-        <v/>
-      </c>
-      <c r="D25" s="7" t="n"/>
+      <c r="C26" s="8">
+        <f>SUM(C5:C25)</f>
+        <v/>
+      </c>
+      <c r="D26" s="7" t="n"/>
+      <c r="E26" s="9">
+        <f>SUM(E5:E25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>Est. Fees</t>
+        </is>
+      </c>
+      <c r="C27" s="15">
+        <f>-E26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="16" t="inlineStr">
+        <is>
+          <t>Net Received</t>
+        </is>
+      </c>
+      <c r="C28" s="17">
+        <f>C26+C27</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1770,13 +2092,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -1786,66 +2109,61 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Fees: Venmo 1.9%+$0.10 · Stripe 2.9%+$0.30 · Check/Zelle free</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Donor</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Mar 24</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>Evan Krakauer</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="n">
-        <v>25</v>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Est. Fee</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>Mar 25</t>
+          <t>Mar 24</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>hallie polsky</t>
+          <t>Evan Krakauer</t>
         </is>
       </c>
       <c r="C5" s="13" t="n">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>0.57</v>
       </c>
     </row>
     <row r="6">
@@ -1856,16 +2174,19 @@
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>Alexa Scalzi</t>
+          <t>hallie polsky</t>
         </is>
       </c>
       <c r="C6" s="13" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>0.78</v>
       </c>
     </row>
     <row r="7">
@@ -1876,16 +2197,19 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Jaimee Manger</t>
+          <t>Alexa Scalzi</t>
         </is>
       </c>
       <c r="C7" s="13" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E7" s="13" t="n">
+        <v>0.67</v>
       </c>
     </row>
     <row r="8">
@@ -1896,16 +2220,19 @@
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>Karen Ganz</t>
+          <t>Jaimee Manger</t>
         </is>
       </c>
       <c r="C8" s="13" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E8" s="13" t="n">
+        <v>0.48</v>
       </c>
     </row>
     <row r="9">
@@ -1916,16 +2243,19 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Debbi Kauffman</t>
+          <t>Karen Ganz</t>
         </is>
       </c>
       <c r="C9" s="13" t="n">
-        <v>100</v>
+        <v>18</v>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>0.44</v>
       </c>
     </row>
     <row r="10">
@@ -1936,16 +2266,19 @@
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>Jan Mirman</t>
+          <t>Debbi Kauffman</t>
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E10" s="13" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -1956,16 +2289,19 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Beth Brody</t>
+          <t>Jan Mirman</t>
         </is>
       </c>
       <c r="C11" s="13" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>1.05</v>
       </c>
     </row>
     <row r="12">
@@ -1976,16 +2312,19 @@
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>Steve Kreinik</t>
+          <t>Beth Brody</t>
         </is>
       </c>
       <c r="C12" s="13" t="n">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>Zelle</t>
-        </is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -1996,30 +2335,82 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
+          <t>Steve Kreinik</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="n">
+        <v>250</v>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Zelle</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
           <t>Eileen Linde</t>
         </is>
       </c>
-      <c r="C13" s="13" t="n">
+      <c r="C14" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="n"/>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n"/>
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C14" s="8">
-        <f>SUM(C4:C13)</f>
-        <v/>
-      </c>
-      <c r="D14" s="7" t="n"/>
+      <c r="C15" s="8">
+        <f>SUM(C5:C14)</f>
+        <v/>
+      </c>
+      <c r="D15" s="7" t="n"/>
+      <c r="E15" s="9">
+        <f>SUM(E5:E14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>Est. Fees</t>
+        </is>
+      </c>
+      <c r="C16" s="15">
+        <f>-E15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Net Received</t>
+        </is>
+      </c>
+      <c r="C17" s="17">
+        <f>C15+C16</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2032,13 +2423,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -2048,45 +2440,37 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Fees: Venmo 1.9%+$0.10 · Stripe 2.9%+$0.30 · Check/Zelle free</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Donor</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>Jason Hornig</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="n">
-        <v>25</v>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Est. Fee</t>
         </is>
       </c>
     </row>
@@ -2098,16 +2482,19 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Meredith Wellen</t>
+          <t>Jason Hornig</t>
         </is>
       </c>
       <c r="C5" s="13" t="n">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>0.57</v>
       </c>
     </row>
     <row r="6">
@@ -2122,12 +2509,15 @@
         </is>
       </c>
       <c r="C6" s="13" t="n">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Venmo</t>
         </is>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>0.78</v>
       </c>
     </row>
     <row r="7">
@@ -2138,30 +2528,82 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
+          <t>Meredith Wellen</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="n">
+        <v>50</v>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="n">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
           <t>Lindsay Koonin</t>
         </is>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C8" s="13" t="n">
         <v>118</v>
       </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="n"/>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="n">
+        <v>2.34</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n"/>
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C8" s="8">
-        <f>SUM(C4:C7)</f>
-        <v/>
-      </c>
-      <c r="D8" s="7" t="n"/>
+      <c r="C9" s="8">
+        <f>SUM(C5:C8)</f>
+        <v/>
+      </c>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="9">
+        <f>SUM(E5:E8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Est. Fees</t>
+        </is>
+      </c>
+      <c r="C10" s="15">
+        <f>-E9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Net Received</t>
+        </is>
+      </c>
+      <c r="C11" s="17">
+        <f>C9+C10</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix Excel formula row alignment; all refs now exact
</commit_message>
<xml_diff>
--- a/Squeeze_Project_Donations.xlsx
+++ b/Squeeze_Project_Donations.xlsx
@@ -91,12 +91,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -497,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fee rates: Venmo 1.9% + $0.10 · Stripe 2.9% + $0.30 · Check/Zelle free</t>
+          <t>Fee rates: Venmo 1.9%+$0.10  ·  Stripe 2.9%+$0.30  ·  Check/Zelle free</t>
         </is>
       </c>
     </row>
@@ -550,21 +551,21 @@
         </is>
       </c>
       <c r="C5" s="4">
-        <f>'Luke &amp; Aria Kerman'!C12</f>
+        <f>'Luke &amp; Aria Kerman'!C13</f>
         <v/>
       </c>
       <c r="D5" s="4">
-        <f>'Luke &amp; Aria Kerman'!C13</f>
-        <v/>
-      </c>
-      <c r="E5" s="4">
-        <f>'Luke &amp; Aria Kerman'!C14</f>
+        <f>'Luke &amp; Aria Kerman'!E13</f>
+        <v/>
+      </c>
+      <c r="E5" s="5">
+        <f>'Luke &amp; Aria Kerman'!C15</f>
         <v/>
       </c>
       <c r="F5" s="4" t="n">
         <v>2250</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="6">
         <f>C5/F5</f>
         <v/>
       </c>
@@ -581,21 +582,21 @@
         </is>
       </c>
       <c r="C6" s="4">
-        <f>'Tessa Forman'!C21</f>
+        <f>'Tessa Forman'!C22</f>
         <v/>
       </c>
       <c r="D6" s="4">
-        <f>'Tessa Forman'!C22</f>
-        <v/>
-      </c>
-      <c r="E6" s="4">
-        <f>'Tessa Forman'!C23</f>
+        <f>'Tessa Forman'!E22</f>
+        <v/>
+      </c>
+      <c r="E6" s="5">
+        <f>'Tessa Forman'!C24</f>
         <v/>
       </c>
       <c r="F6" s="4" t="n">
         <v>2250</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="6">
         <f>C6/F6</f>
         <v/>
       </c>
@@ -612,21 +613,21 @@
         </is>
       </c>
       <c r="C7" s="4">
-        <f>'Ben &amp; Jack'!C25</f>
+        <f>'Ben &amp; Jack'!C26</f>
         <v/>
       </c>
       <c r="D7" s="4">
-        <f>'Ben &amp; Jack'!C26</f>
-        <v/>
-      </c>
-      <c r="E7" s="4">
-        <f>'Ben &amp; Jack'!C27</f>
+        <f>'Ben &amp; Jack'!E26</f>
+        <v/>
+      </c>
+      <c r="E7" s="5">
+        <f>'Ben &amp; Jack'!C28</f>
         <v/>
       </c>
       <c r="F7" s="4" t="n">
         <v>2250</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="6">
         <f>C7/F7</f>
         <v/>
       </c>
@@ -643,21 +644,21 @@
         </is>
       </c>
       <c r="C8" s="4">
-        <f>'Jordana Brody'!C14</f>
+        <f>'Jordana Brody'!C15</f>
         <v/>
       </c>
       <c r="D8" s="4">
-        <f>'Jordana Brody'!C15</f>
-        <v/>
-      </c>
-      <c r="E8" s="4">
-        <f>'Jordana Brody'!C16</f>
+        <f>'Jordana Brody'!E15</f>
+        <v/>
+      </c>
+      <c r="E8" s="5">
+        <f>'Jordana Brody'!C17</f>
         <v/>
       </c>
       <c r="F8" s="4" t="n">
         <v>2250</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="6">
         <f>C8/F8</f>
         <v/>
       </c>
@@ -674,48 +675,48 @@
         </is>
       </c>
       <c r="C9" s="4">
-        <f>'Parker Wellen'!C8</f>
+        <f>'Parker Wellen'!C9</f>
         <v/>
       </c>
       <c r="D9" s="4">
-        <f>'Parker Wellen'!C9</f>
-        <v/>
-      </c>
-      <c r="E9" s="4">
-        <f>'Parker Wellen'!C10</f>
+        <f>'Parker Wellen'!E9</f>
+        <v/>
+      </c>
+      <c r="E9" s="5">
+        <f>'Parker Wellen'!C11</f>
         <v/>
       </c>
       <c r="F9" s="4" t="n">
         <v>2250</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="6">
         <f>C9/F9</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="8">
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="9">
         <f>SUM(C5:C9)</f>
         <v/>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="10">
         <f>SUM(D5:D9)</f>
         <v/>
       </c>
-      <c r="E11" s="8">
+      <c r="E11" s="9">
         <f>SUM(E5:E9)</f>
         <v/>
       </c>
-      <c r="F11" s="9" t="n">
+      <c r="F11" s="10" t="n">
         <v>11250</v>
       </c>
-      <c r="G11" s="10">
+      <c r="G11" s="11">
         <f>C11/F11</f>
         <v/>
       </c>
@@ -742,7 +743,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Luke &amp; Aria Kerman — Camp IHC</t>
         </is>
@@ -751,10 +752,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fees: Venmo 1.9%+$0.10 · Stripe 2.9%+$0.30 · Check/Zelle free</t>
-        </is>
-      </c>
-    </row>
+          <t>Fees: Venmo 1.9%+$0.10  ·  Stripe 2.9%+$0.30  ·  Check/Zelle free</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -783,224 +785,224 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>jayson@license-2-play.com</t>
         </is>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="14" t="n">
         <v>500</v>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
-      <c r="E5" s="13" t="n">
+      <c r="E5" s="14" t="n">
         <v>14.8</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Jarret Kerman</t>
         </is>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
-      <c r="E6" s="13" t="n">
+      <c r="E6" s="14" t="n">
         <v>0.59</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Brooke Jung</t>
         </is>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="D7" s="13" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
-      <c r="E7" s="13" t="n">
+      <c r="E7" s="14" t="n">
         <v>3.2</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Melanie Ringold</t>
         </is>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="14" t="n">
         <v>54</v>
       </c>
-      <c r="D8" s="12" t="inlineStr">
+      <c r="D8" s="13" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
-      <c r="E8" s="13" t="n">
+      <c r="E8" s="14" t="n">
         <v>1.87</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Jarret Kerman</t>
         </is>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="14" t="n">
         <v>200</v>
       </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
-      <c r="E9" s="13" t="n">
+      <c r="E9" s="14" t="n">
         <v>6.1</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Von Maur Foundation</t>
         </is>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" s="14" t="n">
         <v>250</v>
       </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="D10" s="13" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="E10" s="13" t="n">
+      <c r="E10" s="14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>David Brown</t>
         </is>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="D11" s="13" t="inlineStr">
         <is>
           <t>Zelle</t>
         </is>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Craig Brown</t>
         </is>
       </c>
-      <c r="C12" s="13" t="n">
+      <c r="C12" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="n">
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="n">
         <v>1.05</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="A13" s="8" t="n"/>
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="9">
         <f>SUM(C5:C12)</f>
         <v/>
       </c>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="9">
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="10">
         <f>SUM(E5:E12)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>Est. Fees</t>
         </is>
       </c>
-      <c r="C14" s="15">
+      <c r="C14" s="16">
         <f>-E13</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>Net Received</t>
         </is>
       </c>
-      <c r="C15" s="17">
+      <c r="C15" s="18">
         <f>C13+C14</f>
         <v/>
       </c>
@@ -1027,7 +1029,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Tessa Forman — Camp Pontiac</t>
         </is>
@@ -1036,10 +1038,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fees: Venmo 1.9%+$0.10 · Stripe 2.9%+$0.30 · Check/Zelle free</t>
-        </is>
-      </c>
-    </row>
+          <t>Fees: Venmo 1.9%+$0.10  ·  Stripe 2.9%+$0.30  ·  Check/Zelle free</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1068,431 +1071,431 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Allison Slansky</t>
         </is>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="n">
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="n">
         <v>0.57</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Annabelle Greenberg</t>
         </is>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="n">
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="n">
         <v>0.39</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Joshua Henkel</t>
         </is>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="14" t="n">
         <v>36</v>
       </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E7" s="13" t="n">
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="n">
         <v>0.78</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Jen Seiden</t>
         </is>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="14" t="n">
         <v>36</v>
       </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E8" s="13" t="n">
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="n">
         <v>0.78</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Robyn Kreiner</t>
         </is>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="14" t="n">
         <v>36</v>
       </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="n">
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="n">
         <v>0.78</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Erica Polavieja</t>
         </is>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="n">
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="n">
         <v>1.05</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Marissa Drogin</t>
         </is>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="n">
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="n">
         <v>0.57</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Cori Zummo</t>
         </is>
       </c>
-      <c r="C12" s="13" t="n">
+      <c r="C12" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="n">
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="n">
         <v>0.57</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>Lindsey Schnepper</t>
         </is>
       </c>
-      <c r="C13" s="13" t="n">
+      <c r="C13" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E13" s="13" t="n">
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>Christine Schwartz</t>
         </is>
       </c>
-      <c r="C14" s="13" t="n">
+      <c r="C14" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D14" s="13" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
-      <c r="E14" s="13" t="n">
+      <c r="E14" s="14" t="n">
         <v>1.75</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>sarimskier@gmail.com</t>
         </is>
       </c>
-      <c r="C15" s="13" t="n">
+      <c r="C15" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
-      <c r="E15" s="13" t="n">
+      <c r="E15" s="14" t="n">
         <v>1.03</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Jen Schwartz</t>
         </is>
       </c>
-      <c r="C16" s="13" t="n">
+      <c r="C16" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="D16" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E16" s="13" t="n">
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Tracy Paley</t>
         </is>
       </c>
-      <c r="C17" s="13" t="n">
+      <c r="C17" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="D17" s="12" t="inlineStr">
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
-      <c r="E17" s="13" t="n">
+      <c r="E17" s="14" t="n">
         <v>1.75</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>masetheace728@icloud.com</t>
         </is>
       </c>
-      <c r="C18" s="13" t="n">
+      <c r="C18" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="D18" s="12" t="inlineStr">
+      <c r="D18" s="13" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
-      <c r="E18" s="13" t="n">
+      <c r="E18" s="14" t="n">
         <v>0.45</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>Stage to Screen</t>
         </is>
       </c>
-      <c r="C19" s="13" t="n">
+      <c r="C19" s="14" t="n">
         <v>250</v>
       </c>
-      <c r="D19" s="12" t="inlineStr">
+      <c r="D19" s="13" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="E19" s="13" t="n">
+      <c r="E19" s="14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>Rose</t>
         </is>
       </c>
-      <c r="C20" s="13" t="n">
+      <c r="C20" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="D20" s="12" t="inlineStr">
+      <c r="D20" s="13" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="E20" s="13" t="n">
+      <c r="E20" s="14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>Rose</t>
         </is>
       </c>
-      <c r="C21" s="13" t="n">
+      <c r="C21" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="D21" s="12" t="inlineStr">
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="E21" s="13" t="n">
+      <c r="E21" s="14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="n"/>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="A22" s="8" t="n"/>
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C22" s="8">
+      <c r="C22" s="9">
         <f>SUM(C5:C21)</f>
         <v/>
       </c>
-      <c r="D22" s="7" t="n"/>
-      <c r="E22" s="9">
+      <c r="D22" s="8" t="n"/>
+      <c r="E22" s="10">
         <f>SUM(E5:E21)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="14" t="inlineStr">
+      <c r="B23" s="15" t="inlineStr">
         <is>
           <t>Est. Fees</t>
         </is>
       </c>
-      <c r="C23" s="15">
+      <c r="C23" s="16">
         <f>-E22</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="16" t="inlineStr">
+      <c r="B24" s="17" t="inlineStr">
         <is>
           <t>Net Received</t>
         </is>
       </c>
-      <c r="C24" s="17">
+      <c r="C24" s="18">
         <f>C22+C23</f>
         <v/>
       </c>
@@ -1519,7 +1522,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Ben &amp; Jack — Camp Wah-Nee</t>
         </is>
@@ -1528,10 +1531,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fees: Venmo 1.9%+$0.10 · Stripe 2.9%+$0.30 · Check/Zelle free</t>
-        </is>
-      </c>
-    </row>
+          <t>Fees: Venmo 1.9%+$0.10  ·  Stripe 2.9%+$0.30  ·  Check/Zelle free</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1560,523 +1564,523 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Jayson Siano</t>
         </is>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="14" t="n">
         <v>200</v>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
-      <c r="E5" s="13" t="n">
+      <c r="E5" s="14" t="n">
         <v>6.1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Jessica Zipkin</t>
         </is>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="14" t="n">
         <v>150</v>
       </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="n">
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="n">
         <v>2.95</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Stephanie Barilan</t>
         </is>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="14" t="n">
         <v>150</v>
       </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E7" s="13" t="n">
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="n">
         <v>2.95</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Evane Klein</t>
         </is>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E8" s="13" t="n">
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Dana Block</t>
         </is>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="n">
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Jessica Goldstein</t>
         </is>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="n">
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="n">
         <v>1.05</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Jessica Greenwald</t>
         </is>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="n">
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="n">
         <v>1.05</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Jaclyn Vida</t>
         </is>
       </c>
-      <c r="C12" s="13" t="n">
+      <c r="C12" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="n">
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="n">
         <v>1.05</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>Alyse Stern</t>
         </is>
       </c>
-      <c r="C13" s="13" t="n">
+      <c r="C13" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E13" s="13" t="n">
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="n">
         <v>1.05</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>ali horowitz</t>
         </is>
       </c>
-      <c r="C14" s="13" t="n">
+      <c r="C14" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="D14" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E14" s="13" t="n">
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="n">
         <v>1.05</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Dina Goldberg</t>
         </is>
       </c>
-      <c r="C15" s="13" t="n">
+      <c r="C15" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E15" s="13" t="n">
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="n">
         <v>1.05</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Liz Beler</t>
         </is>
       </c>
-      <c r="C16" s="13" t="n">
+      <c r="C16" s="14" t="n">
         <v>40</v>
       </c>
-      <c r="D16" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E16" s="13" t="n">
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="n">
         <v>0.86</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Elizabeth Zorn</t>
         </is>
       </c>
-      <c r="C17" s="13" t="n">
+      <c r="C17" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="D17" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E17" s="13" t="n">
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="n">
         <v>0.57</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>Michael Jacobson</t>
         </is>
       </c>
-      <c r="C18" s="13" t="n">
+      <c r="C18" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="D18" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E18" s="13" t="n">
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="n">
         <v>0.57</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>Erica Oliver</t>
         </is>
       </c>
-      <c r="C19" s="13" t="n">
+      <c r="C19" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="D19" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E19" s="13" t="n">
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="n">
         <v>0.57</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>Robyn Sachnoff</t>
         </is>
       </c>
-      <c r="C20" s="13" t="n">
+      <c r="C20" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="D20" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E20" s="13" t="n">
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="n">
         <v>0.57</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>Jennifer Brogadir</t>
         </is>
       </c>
-      <c r="C21" s="13" t="n">
+      <c r="C21" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="D21" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E21" s="13" t="n">
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="n">
         <v>0.48</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Ellen Jacobson</t>
         </is>
       </c>
-      <c r="C22" s="13" t="n">
+      <c r="C22" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E22" s="13" t="n">
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="n">
         <v>0.57</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Joey Stella</t>
         </is>
       </c>
-      <c r="C23" s="13" t="n">
+      <c r="C23" s="14" t="n">
         <v>200</v>
       </c>
-      <c r="D23" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E23" s="13" t="n">
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="n">
         <v>3.9</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>Carrie Grochow</t>
         </is>
       </c>
-      <c r="C24" s="13" t="n">
+      <c r="C24" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="D24" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E24" s="13" t="n">
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
         <is>
           <t>Rebecca Brogadir</t>
         </is>
       </c>
-      <c r="C25" s="13" t="n">
+      <c r="C25" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="D25" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E25" s="13" t="n">
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="n"/>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="A26" s="8" t="n"/>
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C26" s="8">
+      <c r="C26" s="9">
         <f>SUM(C5:C25)</f>
         <v/>
       </c>
-      <c r="D26" s="7" t="n"/>
-      <c r="E26" s="9">
+      <c r="D26" s="8" t="n"/>
+      <c r="E26" s="10">
         <f>SUM(E5:E25)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="14" t="inlineStr">
+      <c r="B27" s="15" t="inlineStr">
         <is>
           <t>Est. Fees</t>
         </is>
       </c>
-      <c r="C27" s="15">
+      <c r="C27" s="16">
         <f>-E26</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="16" t="inlineStr">
+      <c r="B28" s="17" t="inlineStr">
         <is>
           <t>Net Received</t>
         </is>
       </c>
-      <c r="C28" s="17">
+      <c r="C28" s="18">
         <f>C26+C27</f>
         <v/>
       </c>
@@ -2103,7 +2107,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Jordana Brody — Camp Westmont</t>
         </is>
@@ -2112,10 +2116,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fees: Venmo 1.9%+$0.10 · Stripe 2.9%+$0.30 · Check/Zelle free</t>
-        </is>
-      </c>
-    </row>
+          <t>Fees: Venmo 1.9%+$0.10  ·  Stripe 2.9%+$0.30  ·  Check/Zelle free</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2144,270 +2149,270 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Mar 24</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Evan Krakauer</t>
         </is>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="n">
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="n">
         <v>0.57</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>hallie polsky</t>
         </is>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="14" t="n">
         <v>36</v>
       </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="n">
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="n">
         <v>0.78</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Alexa Scalzi</t>
         </is>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="14" t="n">
         <v>30</v>
       </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E7" s="13" t="n">
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="n">
         <v>0.67</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Jaimee Manger</t>
         </is>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E8" s="13" t="n">
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="n">
         <v>0.48</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Karen Ganz</t>
         </is>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="14" t="n">
         <v>18</v>
       </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="n">
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="n">
         <v>0.44</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Debbi Kauffman</t>
         </is>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="n">
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Jan Mirman</t>
         </is>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="n">
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="n">
         <v>1.05</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Beth Brody</t>
         </is>
       </c>
-      <c r="C12" s="13" t="n">
+      <c r="C12" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="n">
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>Steve Kreinik</t>
         </is>
       </c>
-      <c r="C13" s="13" t="n">
+      <c r="C13" s="14" t="n">
         <v>250</v>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
         <is>
           <t>Zelle</t>
         </is>
       </c>
-      <c r="E13" s="13" t="n">
+      <c r="E13" s="14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>Eileen Linde</t>
         </is>
       </c>
-      <c r="C14" s="13" t="n">
+      <c r="C14" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="D14" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E14" s="13" t="n">
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n"/>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="A15" s="8" t="n"/>
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C15" s="8">
+      <c r="C15" s="9">
         <f>SUM(C5:C14)</f>
         <v/>
       </c>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="9">
+      <c r="D15" s="8" t="n"/>
+      <c r="E15" s="10">
         <f>SUM(E5:E14)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="14" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t>Est. Fees</t>
         </is>
       </c>
-      <c r="C16" s="15">
+      <c r="C16" s="16">
         <f>-E15</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>Net Received</t>
         </is>
       </c>
-      <c r="C17" s="17">
+      <c r="C17" s="18">
         <f>C15+C16</f>
         <v/>
       </c>
@@ -2434,7 +2439,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Parker Wellen — Camp Pontiac</t>
         </is>
@@ -2443,10 +2448,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fees: Venmo 1.9%+$0.10 · Stripe 2.9%+$0.30 · Check/Zelle free</t>
-        </is>
-      </c>
-    </row>
+          <t>Fees: Venmo 1.9%+$0.10  ·  Stripe 2.9%+$0.30  ·  Check/Zelle free</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2475,132 +2481,132 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Jason Hornig</t>
         </is>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="n">
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="n">
         <v>0.57</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Meredith Wellen</t>
         </is>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="14" t="n">
         <v>36</v>
       </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="n">
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="n">
         <v>0.78</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Meredith Wellen</t>
         </is>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E7" s="13" t="n">
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="n">
         <v>1.05</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Mar 25</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Lindsay Koonin</t>
         </is>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="14" t="n">
         <v>118</v>
       </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>Venmo</t>
-        </is>
-      </c>
-      <c r="E8" s="13" t="n">
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="n">
         <v>2.34</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="A9" s="8" t="n"/>
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="9">
         <f>SUM(C5:C8)</f>
         <v/>
       </c>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="9">
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="10">
         <f>SUM(E5:E8)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>Est. Fees</t>
         </is>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="16">
         <f>-E9</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>Net Received</t>
         </is>
       </c>
-      <c r="C11" s="17">
+      <c r="C11" s="18">
         <f>C9+C10</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Alison Enis \$20 → Ben & Jack; raised \$1,605; ticker \$4,855
</commit_message>
<xml_diff>
--- a/Squeeze_Project_Donations.xlsx
+++ b/Squeeze_Project_Donations.xlsx
@@ -756,7 +756,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1042,7 +1041,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1511,7 +1509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2047,40 +2045,63 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="n"/>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>Alison Enis</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="n">
+        <v>0.48</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="n"/>
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C26" s="9">
+      <c r="C27" s="9">
         <f>SUM(C5:C25)</f>
         <v/>
       </c>
-      <c r="D26" s="8" t="n"/>
-      <c r="E26" s="10">
+      <c r="D27" s="8" t="n"/>
+      <c r="E27" s="10">
         <f>SUM(E5:E25)</f>
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="15" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="15" t="inlineStr">
         <is>
           <t>Est. Fees</t>
         </is>
       </c>
-      <c r="C27" s="16">
+      <c r="C28" s="16">
         <f>-E26</f>
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="17" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="17" t="inlineStr">
         <is>
           <t>Net Received</t>
         </is>
       </c>
-      <c r="C28" s="18">
+      <c r="C29" s="18">
         <f>C26+C27</f>
         <v/>
       </c>
@@ -2120,7 +2141,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2452,7 +2472,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Kevin Saliba \$100 Stripe → Luke & Aria; raised \$1,364; ticker \$4,970
</commit_message>
<xml_diff>
--- a/Squeeze_Project_Donations.xlsx
+++ b/Squeeze_Project_Donations.xlsx
@@ -732,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -756,6 +756,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -968,40 +969,63 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="n"/>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Kevin Saliba</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n"/>
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C13" s="9">
+      <c r="C14" s="9">
         <f>SUM(C5:C12)</f>
         <v/>
       </c>
-      <c r="D13" s="8" t="n"/>
-      <c r="E13" s="10">
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="10">
         <f>SUM(E5:E12)</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="15" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>Est. Fees</t>
         </is>
       </c>
-      <c r="C14" s="16">
+      <c r="C15" s="16">
         <f>-E13</f>
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="B15" s="17" t="inlineStr">
+    <row r="16">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>Net Received</t>
         </is>
       </c>
-      <c r="C15" s="18">
+      <c r="C16" s="18">
         <f>C13+C14</f>
         <v/>
       </c>
@@ -1533,7 +1557,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>

</xml_diff>